<commit_message>
Mensagem do que alteraste
</commit_message>
<xml_diff>
--- a/medicamentos.xlsx
+++ b/medicamentos.xlsx
@@ -2316,7 +2316,7 @@
     <t>A02BA03</t>
   </si>
   <si>
-    <t>Imagens/Generic.webp</t>
+    <t>Imagens/MSRM.png</t>
   </si>
   <si>
     <t>Cytotec</t>
@@ -12661,7 +12661,7 @@
       <c r="AB54" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="AC54" s="1" t="s">
+      <c r="AC54" s="15" t="s">
         <v>535</v>
       </c>
       <c r="AD54" s="7" t="s">

</xml_diff>